<commit_message>
Clarify hosting scope: AWS Commercial, us-east-2
- SDR v1.2: MAS-CSO-IIR names AWS Commercial us-east-2 as the hosting
  environment and excludes other regions (including Europe) and the
  AWS GovCloud (US) proof of concept
- SDR: backups described as replicated across availability zones
  (MAS-CSO-IIR, KSI-SVC-SIN), matching the SOC 2 description
- Public Information JSON and readable version: replace 'dedicated
  environment' wording with hosting location

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QqdRwbgxpbgZLeo3nnYUym
</commit_message>
<xml_diff>
--- a/JupiterOne_FedRAMP_ClassA_Security_Decision_Record.xlsx
+++ b/JupiterOne_FedRAMP_ClassA_Security_Decision_Record.xlsx
@@ -893,10 +893,10 @@
       <c r="G8" s="28" t="inlineStr">
         <is>
           <t>JupiterOne GovCloud (the cloud service offering) is defined as the set of information resources that handle federal customer data or are likely to impact the confidentiality, integrity, or availability of federal customer data. The set was identified by tracing where federal customer data is stored, processed, and transmitted, and which resources administer, monitor, build, or deploy those components.
-Resources that handle federal customer data: the JupiterOne GovCloud application and API services; the AWS compute, storage, and database services that host them; AWS networking (VPC, security groups, load balancing, WAF); encrypted backups replicated between AWS regions; and metadata about federal customer data generated by these services.
+Resources that handle federal customer data: the JupiterOne GovCloud application and API services, hosted in AWS Commercial in the us-east-2 region; the AWS compute, storage, and database services that host them; AWS networking (VPC, security groups, load balancing, WAF); encrypted backups replicated across multiple availability zones within us-east-2; and metadata about federal customer data generated by these services.
 Resources likely to impact federal customer data: staff identity and access management (single sign-on identity provider, hardware security keys, VPN); the CI/CD pipeline and version control that deliver code to production; logging, monitoring, and SIEM tooling (AWS CloudWatch, Panther); and vulnerability scanning tooling.
-Third-party information resources: Amazon Web Services is the underlying infrastructure provider, as listed under thirdPartyInformationResources in the Public Information JSON. Atlassian Statuspage hosts the public status page and does not handle federal customer data.
-Excluded: JupiterOne's commercial (non-GovCloud) environment and corporate business systems that neither handle federal customer data nor have access that could affect the GovCloud environment.</t>
+Third-party information resources: Amazon Web Services (AWS Commercial, us-east-2) is the underlying infrastructure provider, as listed under thirdPartyInformationResources in the Public Information JSON. Atlassian Statuspage hosts the public status page and does not handle federal customer data.
+Excluded: JupiterOne production deployments in AWS regions other than us-east-2, including Europe, which serve non-federal customers and are not part of this offering; a proof-of-concept environment in AWS GovCloud (US), which has no users or federal data; and corporate business systems that neither handle federal customer data nor have access that could affect the offering.</t>
         </is>
       </c>
       <c r="H8" s="28" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="N8" s="28" t="inlineStr">
         <is>
-          <t>Rewritten 2026-10-30 per FedRAMP feedback to address the rule directly rather than referencing the SOC 2 system description.</t>
+          <t>Rewritten 2026-10-30 per FedRAMP feedback to address the rule directly; hosting scope (AWS Commercial, us-east-2) clarified.</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="G27" s="28" t="inlineStr">
         <is>
-          <t>AES-256 encryption at rest; TLS with trusted CA certificates in transit; encrypted backup replication between cloud regions.</t>
+          <t>AES-256 encryption at rest; TLS with trusted CA certificates in transit; encrypted backups replicated across multiple availability zones.</t>
         </is>
       </c>
       <c r="H27" s="28" t="inlineStr">
@@ -2968,7 +2968,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="22">
       <c r="A3" s="33" t="inlineStr">
         <is>
@@ -3036,7 +3035,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="22">
       <c r="A9" s="33" t="inlineStr">
         <is>
@@ -3104,7 +3102,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="39" t="inlineStr">
         <is>

</xml_diff>